<commit_message>
termine el template de la vista step2
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45163.60820518518</v>
+        <v>45214</v>
       </c>
     </row>
     <row r="2">
@@ -844,7 +844,7 @@
       </c>
       <c r="C26" s="20" t="n"/>
       <c r="D26" s="22" t="n">
-        <v>633.7786400000001</v>
+        <v>602.352</v>
       </c>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="23" t="n"/>
@@ -863,7 +863,7 @@
       </c>
       <c r="C27" s="20" t="n"/>
       <c r="D27" s="22" t="n">
-        <v>50000</v>
+        <v>602.352</v>
       </c>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
@@ -882,7 +882,7 @@
       </c>
       <c r="C28" s="20" t="n"/>
       <c r="D28" s="22" t="n">
-        <v>305.67</v>
+        <v>709.045</v>
       </c>
       <c r="E28" s="23" t="n"/>
       <c r="F28" s="23" t="n"/>
@@ -901,7 +901,7 @@
       </c>
       <c r="C29" s="20" t="n"/>
       <c r="D29" s="22" t="n">
-        <v>528.38</v>
+        <v>1225.63</v>
       </c>
       <c r="E29" s="23" t="n"/>
       <c r="F29" s="23" t="n"/>
@@ -920,7 +920,7 @@
       </c>
       <c r="C30" s="20" t="n"/>
       <c r="D30" s="22" t="n">
-        <v>651.92</v>
+        <v>1512.193</v>
       </c>
       <c r="E30" s="23" t="n"/>
       <c r="F30" s="23" t="n"/>
@@ -939,7 +939,7 @@
       </c>
       <c r="C31" s="20" t="n"/>
       <c r="D31" s="22" t="n">
-        <v>864.72</v>
+        <v>2005.801</v>
       </c>
       <c r="E31" s="23" t="n"/>
       <c r="F31" s="23" t="n"/>
@@ -958,7 +958,7 @@
       </c>
       <c r="C32" s="20" t="n"/>
       <c r="D32" s="22" t="n">
-        <v>1229.9</v>
+        <v>2852.872</v>
       </c>
       <c r="E32" s="23" t="n"/>
       <c r="F32" s="23" t="n"/>
@@ -977,7 +977,7 @@
       </c>
       <c r="C33" s="20" t="n"/>
       <c r="D33" s="22" t="n">
-        <v>1821.4</v>
+        <v>4224.918</v>
       </c>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="23" t="n"/>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C35" s="20" t="n"/>
       <c r="D35" s="22" t="n">
-        <v>383.21</v>
+        <v>888.897</v>
       </c>
       <c r="E35" s="23" t="n"/>
       <c r="F35" s="23" t="n"/>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C36" s="20" t="n"/>
       <c r="D36" s="22" t="n">
-        <v>433.71</v>
+        <v>1006.036</v>
       </c>
       <c r="E36" s="23" t="n"/>
       <c r="F36" s="23" t="n"/>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="C37" s="20" t="n"/>
       <c r="D37" s="22" t="n">
-        <v>553.63</v>
+        <v>1284.213</v>
       </c>
       <c r="E37" s="23" t="n"/>
       <c r="F37" s="23" t="n"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="C38" s="20" t="n"/>
       <c r="D38" s="22" t="n">
-        <v>919.72</v>
+        <v>2133.396</v>
       </c>
       <c r="E38" s="23" t="n"/>
       <c r="F38" s="23" t="n"/>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C39" s="20" t="n"/>
       <c r="D39" s="22" t="n">
-        <v>1192.92</v>
+        <v>2767.105</v>
       </c>
       <c r="E39" s="23" t="n"/>
       <c r="F39" s="23" t="n"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C40" s="20" t="n"/>
       <c r="D40" s="22" t="n">
-        <v>1521.13</v>
+        <v>3528.424</v>
       </c>
       <c r="E40" s="23" t="n"/>
       <c r="F40" s="23" t="n"/>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C41" s="20" t="n"/>
       <c r="D41" s="22" t="n">
-        <v>2138.79</v>
+        <v>4961.133</v>
       </c>
       <c r="E41" s="23" t="n"/>
       <c r="F41" s="23" t="n"/>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C42" s="20" t="n"/>
       <c r="D42" s="22" t="n">
-        <v>3300.15</v>
+        <v>7655.029</v>
       </c>
       <c r="E42" s="23" t="n"/>
       <c r="F42" s="23" t="n"/>

</xml_diff>

<commit_message>
funcionalidad de porcentaje negativa, para todos el mismo porcentaje
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45214</v>
+        <v>45216</v>
       </c>
     </row>
     <row r="2">
@@ -863,7 +863,7 @@
       </c>
       <c r="C27" s="20" t="n"/>
       <c r="D27" s="22" t="n">
-        <v>602.352</v>
+        <v>700</v>
       </c>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>

</xml_diff>

<commit_message>
arreglando bug de la autodeteccion
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45217</v>
+        <v>45219</v>
       </c>
     </row>
     <row r="2">
@@ -844,7 +844,7 @@
       </c>
       <c r="C26" s="20" t="n"/>
       <c r="D26" s="22" t="n">
-        <v>542.1168</v>
+        <v>602.352</v>
       </c>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="23" t="n"/>
@@ -863,7 +863,7 @@
       </c>
       <c r="C27" s="20" t="n"/>
       <c r="D27" s="22" t="n">
-        <v>630</v>
+        <v>700</v>
       </c>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
@@ -882,7 +882,7 @@
       </c>
       <c r="C28" s="20" t="n"/>
       <c r="D28" s="22" t="n">
-        <v>638.1405</v>
+        <v>709.045</v>
       </c>
       <c r="E28" s="23" t="n"/>
       <c r="F28" s="23" t="n"/>
@@ -901,7 +901,7 @@
       </c>
       <c r="C29" s="20" t="n"/>
       <c r="D29" s="22" t="n">
-        <v>1103.067</v>
+        <v>1225.63</v>
       </c>
       <c r="E29" s="23" t="n"/>
       <c r="F29" s="23" t="n"/>
@@ -920,7 +920,7 @@
       </c>
       <c r="C30" s="20" t="n"/>
       <c r="D30" s="22" t="n">
-        <v>1360.9737</v>
+        <v>1512.193</v>
       </c>
       <c r="E30" s="23" t="n"/>
       <c r="F30" s="23" t="n"/>
@@ -939,7 +939,7 @@
       </c>
       <c r="C31" s="20" t="n"/>
       <c r="D31" s="22" t="n">
-        <v>1805.2209</v>
+        <v>2005.801</v>
       </c>
       <c r="E31" s="23" t="n"/>
       <c r="F31" s="23" t="n"/>
@@ -958,7 +958,7 @@
       </c>
       <c r="C32" s="20" t="n"/>
       <c r="D32" s="22" t="n">
-        <v>2567.5848</v>
+        <v>2852.872</v>
       </c>
       <c r="E32" s="23" t="n"/>
       <c r="F32" s="23" t="n"/>
@@ -977,7 +977,7 @@
       </c>
       <c r="C33" s="20" t="n"/>
       <c r="D33" s="22" t="n">
-        <v>3802.4262</v>
+        <v>4224.918</v>
       </c>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="23" t="n"/>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="C35" s="20" t="n"/>
       <c r="D35" s="22" t="n">
-        <v>800.0073</v>
+        <v>888.897</v>
       </c>
       <c r="E35" s="23" t="n"/>
       <c r="F35" s="23" t="n"/>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C36" s="20" t="n"/>
       <c r="D36" s="22" t="n">
-        <v>905.4323999999999</v>
+        <v>1006.036</v>
       </c>
       <c r="E36" s="23" t="n"/>
       <c r="F36" s="23" t="n"/>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="C37" s="20" t="n"/>
       <c r="D37" s="22" t="n">
-        <v>1155.7917</v>
+        <v>1284.213</v>
       </c>
       <c r="E37" s="23" t="n"/>
       <c r="F37" s="23" t="n"/>
@@ -1074,7 +1074,7 @@
       </c>
       <c r="C38" s="20" t="n"/>
       <c r="D38" s="22" t="n">
-        <v>1920.0564</v>
+        <v>2133.396</v>
       </c>
       <c r="E38" s="23" t="n"/>
       <c r="F38" s="23" t="n"/>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="C39" s="20" t="n"/>
       <c r="D39" s="22" t="n">
-        <v>2490.3945</v>
+        <v>2767.105</v>
       </c>
       <c r="E39" s="23" t="n"/>
       <c r="F39" s="23" t="n"/>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C40" s="20" t="n"/>
       <c r="D40" s="22" t="n">
-        <v>3175.5816</v>
+        <v>3528.424</v>
       </c>
       <c r="E40" s="23" t="n"/>
       <c r="F40" s="23" t="n"/>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C41" s="20" t="n"/>
       <c r="D41" s="22" t="n">
-        <v>4465.0197</v>
+        <v>4961.133</v>
       </c>
       <c r="E41" s="23" t="n"/>
       <c r="F41" s="23" t="n"/>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C42" s="20" t="n"/>
       <c r="D42" s="22" t="n">
-        <v>6889.5261</v>
+        <v>7655.029</v>
       </c>
       <c r="E42" s="23" t="n"/>
       <c r="F42" s="23" t="n"/>
@@ -1182,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A12:D12"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
haciendo el drive pero con fallos
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45223</v>
+        <v>45230</v>
       </c>
     </row>
     <row r="2">
@@ -1182,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B42:C42"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
resolvbiendo el problea al subir al drive y guardar los cambios de los archivo en la base de datos
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45234</v>
+        <v>45236</v>
       </c>
     </row>
     <row r="2">
@@ -863,7 +863,7 @@
       </c>
       <c r="C27" s="20" t="n"/>
       <c r="D27" s="22" t="n">
-        <v>700</v>
+        <v>680</v>
       </c>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
@@ -1182,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A12:D12"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
subido al drive arreglado. Falta pulir codigo y testing + crud del drive y listats
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45236</v>
+        <v>45237</v>
       </c>
     </row>
     <row r="2">
@@ -1182,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B42:C42"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
file dravie corriptos con el id ddel drive
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45237</v>
+        <v>45238</v>
       </c>
     </row>
     <row r="2">
@@ -1182,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A12:D12"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
error al agregar articulo automaticamente resuelto
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45256</v>
+        <v>45261</v>
       </c>
     </row>
     <row r="2">
@@ -1182,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A12:D12"/>
     <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
fucionalidad testing prices auto echa y correcion de errores y redundacia quitando la carpeta listas_ordenadas del sistema
</commit_message>
<xml_diff>
--- a/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/ma/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45261</v>
+        <v>45266</v>
       </c>
     </row>
     <row r="2">
@@ -1182,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B42:C42"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>